<commit_message>
투자 대시보드 2026-10-14 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-10-13.xlsx
+++ b/technicals/exports/2026-10-13.xlsx
@@ -142,7 +142,7 @@
       </ns0:c>
       <ns0:c r="F2" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 스마트폰, 개인용 컴퓨터, 태블릿, 웨어러블 및 액세서리를 설계·제조·판매.</ns0:t>
+          <ns0:t>전 세계에서 스마트폰·PC·태블릿·웨어러블·액세서리를 설계·제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G2">
@@ -221,7 +221,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 의약품과 치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
+          <ns0:t>전 세계에서 의약품·치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
@@ -300,7 +300,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 건설·엔지니어링 구조물·운송 시장에 인프라 관련 제품과 솔루션을 제공한다.</ns0:t>
+          <ns0:t>미국 건설·엔지니어링 구조물·운송 시장에 인프라 제품과 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -379,7 +379,7 @@
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>미주·유럽·중동·아시아 등에서 소비자용, 학교용, 기술 및 사무용 제품을 설계·제조·판매.</ns0:t>
+          <ns0:t>미주·유럽·중동·아시아 등에서 소비자·학교·기술·사무용 제품을 설계·제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5">
@@ -458,7 +458,7 @@
       </ns0:c>
       <ns0:c r="F6" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·이집트·북해에서 천연가스, 원유 및 천연가스액을 탐사·개발·생산하는 독립 에너지 기업.</ns0:t>
+          <ns0:t>미국·이집트·북해에서 천연가스·원유·천연가스액을 탐사·개발·생산하는 독립 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G6">
@@ -537,7 +537,7 @@
       </ns0:c>
       <ns0:c r="F7" t="inlineStr">
         <ns0:is>
-          <ns0:t>북미·유럽 등에서 온라인 데이팅·소셜 네트워킹 앱을 운영하며 구독과 앱 내 구매를 제공.</ns0:t>
+          <ns0:t>북미·유럽 등에서 데이팅·소셜 네트워킹 앱을 운영하며 구독과 앱 내 구매 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G7">
@@ -616,7 +616,7 @@
       </ns0:c>
       <ns0:c r="F8" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 석유·가스 사업을 운영하며 가스·저탄소 에너지, 석유 생산 및 고객·제품 부문을 영위.</ns0:t>
+          <ns0:t>전 세계에서 가스·저탄소 에너지, 석유 생산, 고객·제품 부문 등 석유·가스 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G8">
@@ -695,7 +695,7 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료기술 기업으로 급성기 환자용 현장 뇌파검사 플랫폼인 Ceribell System을 개발.</ns0:t>
+          <ns0:t>급성기 환자용 현장 뇌파검사 플랫폼 Ceribell System을 개발하는 미국 의료기술 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9">
@@ -932,7 +932,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 보험 보장이 부족한 가정과 기업에 프로그램·서비스를 제공하는 관리형 의료 기업.</ns0:t>
+          <ns0:t>미국 내 보험 보장이 부족한 가정·기업에 프로그램과 서비스를 제공하는 관리형 의료 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1011,7 +1011,7 @@
       </ns0:c>
       <ns0:c r="F13" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·공공부문 등에 컴퓨터 시스템과 데이터센터를 포함한 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>기업·공공부문에 컴퓨터 시스템·데이터센터 등 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G13">
@@ -1090,7 +1090,7 @@
       </ns0:c>
       <ns0:c r="F14" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소 등을 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
+          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소를 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G14">
@@ -1169,7 +1169,7 @@
       </ns0:c>
       <ns0:c r="F15" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 재생연료, 석유 정제·판매 및 질소비료 제조 사업을 영위하는 기업.</ns0:t>
+          <ns0:t>미국에서 재생연료, 석유 정제·판매, 질소비료 제조 사업을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G15">
@@ -1248,7 +1248,7 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유·천연가스 탐사, 개발, 생산, 운송 등을 포함한 통합 에너지 및 화학 사업을 영위.</ns0:t>
+          <ns0:t>원유·천연가스 탐사·개발·생산·운송 등을 포함한 통합 에너지·화학 사업 영위.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16">
@@ -1327,7 +1327,7 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>한국·미국 등에서 캐주얼 게임과 모바일 앱을 개발·배급하며 소셜 카지노 게임 및 iGaming 사업 운영.</ns0:t>
+          <ns0:t>한국·미국 등에서 캐주얼 게임·모바일 앱을 개발·배급하고 소셜 카지노와 iGaming 사업을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17">
@@ -1406,7 +1406,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하며 기술 관리 서비스도 제공하는 기업.</ns0:t>
+          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하고 기술 관리 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1485,7 +1485,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 독립 에너지 기업으로 정유·재생에너지·마케팅·윤활유·미드스트림 사업과 연료 생산·판매를 수행.</ns0:t>
+          <ns0:t>미국 독립 에너지 기업으로 정유·재생에너지·윤활유·미드스트림 사업과 연료 생산·판매 수행.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1564,7 +1564,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>디지털 기업의 복잡한 디지털 환경을 위한 AI 기반 관측성 플랫폼을 제공하는 기업.</ns0:t>
+          <ns0:t>기업의 복잡한 디지털 환경을 위한 AI 기반 관측성 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1722,7 +1722,7 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 부실 소비자 채권을 할인 매입·관리하며 채무 회수 솔루션과 관련 서비스를 제공.</ns0:t>
+          <ns0:t>전 세계 부실 소비자 채권을 할인 매입·관리하며 채무 회수 솔루션과 관련 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22">
@@ -1880,7 +1880,7 @@
       </ns0:c>
       <ns0:c r="F24" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 의료용 의류, 신발 등 생활용품을 소비자에게 직접 판매하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 의료용 의류·신발 등 생활용품을 소비자에게 직접 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24">
@@ -1959,7 +1959,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>시계·스마트워치·주얼리·핸드백·가죽 소품·벨트·선글라스 등 패션 액세서리를 설계·개발·유통.</ns0:t>
+          <ns0:t>시계·스마트워치·주얼리·핸드백·가죽 소품·벨트·선글라스 등 패션 액세서리 설계·개발·유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2038,7 +2038,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 초대형 원유운반선, 수에즈막스, LR2·아프라막스 등 원유·석유제품 운반선을 보유·운영.</ns0:t>
+          <ns0:t>전 세계에서 초대형·수에즈막스·LR2·아프라막스 원유·석유제품 운반선 보유·운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2117,7 +2117,7 @@
       </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 사이버보안 및 네트워크·보안 통합 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>전 세계에 사이버보안과 네트워크·보안 통합 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G27">
@@ -2275,7 +2275,7 @@
       </ns0:c>
       <ns0:c r="F29" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임, 수집품, 엔터테인먼트 제품을 판매하는 기업.</ns0:t>
+          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임·수집품·엔터테인먼트 제품을 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29">
@@ -2354,7 +2354,7 @@
       </ns0:c>
       <ns0:c r="F30" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 및 해외에서 에너지 서비스를 제공하며 전력·천연가스 재판매와 재생에너지 사업을 영위.</ns0:t>
+          <ns0:t>미국 및 해외에서 전력·천연가스 재판매와 재생에너지 등 에너지 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G30">
@@ -2433,7 +2433,7 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>소프트웨어 개발 전 과정을 지원하는 통합 DevSecOps 플랫폼 GitLab을 제공하는 기업.</ns0:t>
+          <ns0:t>소프트웨어 개발 전 과정을 지원하는 통합 DevSecOps 플랫폼 GitLab을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31">
@@ -2512,7 +2512,7 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>혈장·혈액센터·병원 부문의 의료기술 기업으로 자동 혈장 채취 시스템과 헌혈자 관리 소프트웨어 등을 제공.</ns0:t>
+          <ns0:t>혈장·혈액센터·병원용 의료기술 기업으로 자동 혈장 채취 시스템과 헌혈자 관리 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32">
@@ -2591,7 +2591,7 @@
       </ns0:c>
       <ns0:c r="F33" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험을 제공하며 보험·마켓플레이스 부문을 운영.</ns0:t>
+          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험과 마켓플레이스 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G33">
@@ -2670,7 +2670,7 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국과 해외에서 다양한 형태의 맞춤형 냉간 성형 강재를 제조·판매하는 회사.</ns0:t>
+          <ns0:t>중국과 해외에서 다양한 맞춤형 냉간 성형 강재를 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34">
@@ -2749,7 +2749,7 @@
       </ns0:c>
       <ns0:c r="F35" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술로 의료 제공을 확장·자동화하며 급성 부상·만성 통증·수술 후 재활 등 근골격계 관리 플랫폼을 개발하는 기업.</ns0:t>
+          <ns0:t>급성 부상·만성 통증·수술 후 재활 등 근골격계 관리를 위한 의료 자동화 플랫폼 개발 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G35">
@@ -2907,7 +2907,7 @@
       </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료기관에 SaaS 애플리케이션과 의료 제공자 채용·신청·면허 검증 등 관리 도구를 제공.</ns0:t>
+          <ns0:t>미국 의료기관에 SaaS와 의료 제공자 채용·신청·면허 검증 관리 도구를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G37">
@@ -2986,7 +2986,7 @@
       </ns0:c>
       <ns0:c r="F38" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공하는 기업.</ns0:t>
+          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G38">
@@ -3065,7 +3065,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 소비재 브랜드 등의 디지털 판촉을 제휴 매체 네트워크를 통해 소비자에게 제공.</ns0:t>
+          <ns0:t>미국 소비재 브랜드 등의 디지털 판촉을 제휴 매체 네트워크로 소비자에게 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3144,7 +3144,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3223,7 +3223,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>싱가포르·동남아에서 재생·신규 용기를 판매하고 강철·플라스틱 드럼 등 용기 재생 서비스를 제공.</ns0:t>
+          <ns0:t>싱가포르·동남아에서 재생·신규 용기를 판매하고 강철·플라스틱 드럼 등의 재생 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3299,7 +3299,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>소셜 서비스와 통신 기술을 제공하며 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영한다.</ns0:t>
+          <ns0:t>소셜 서비스·통신 기술을 제공하고 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3457,7 +3457,7 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44">
@@ -3533,7 +3533,7 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>맞춤형 선박을 활용한 해양 탐험과 육상 여행 체험을 전 세계에 제공하는 기업.</ns0:t>
+          <ns0:t>맞춤형 선박을 활용한 해양 탐험과 육상 여행 체험을 전 세계에 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45">
@@ -3612,7 +3612,7 @@
       </ns0:c>
       <ns0:c r="F46" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 거래 처리 및 결제 관련 제품·서비스를 소비자, 가맹점, 금융기관 등에 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 소비자·가맹점·금융기관 등에 거래 처리와 결제 제품·서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G46">
@@ -3691,7 +3691,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 보험, 연금, 임직원 복리후생 및 자산관리 서비스를 제공하는 금융서비스 기업.</ns0:t>
+          <ns0:t>전 세계에서 보험·연금·임직원 복리후생·자산관리 서비스를 제공하는 금융서비스 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">
@@ -3770,7 +3770,7 @@
       </ns0:c>
       <ns0:c r="F48" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국의 통합 다운스트림 에너지 기업으로 정유·판매, 미드스트림, 재생 디젤 사업을 운영한다.</ns0:t>
+          <ns0:t>미국에서 정유·판매, 미드스트림, 재생 디젤 사업을 운영하는 통합 다운스트림 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G48">
@@ -3849,7 +3849,7 @@
       </ns0:c>
       <ns0:c r="F49" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·멕시코·영국 등에서 금속가공 및 유지보수·수리·운영용 제품과 서비스를 유통한다.</ns0:t>
+          <ns0:t>미국·캐나다·멕시코·영국 등에서 금속가공 및 유지보수·수리·운영용 제품과 서비스를 유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G49">
@@ -3928,7 +3928,7 @@
       </ns0:c>
       <ns0:c r="F50" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
+          <ns0:t>전 세계에 실험실용 기기 등 정밀기기를 제조·공급하고 관련 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G50">
@@ -4007,7 +4007,7 @@
       </ns0:c>
       <ns0:c r="F51" t="inlineStr">
         <ns0:is>
-          <ns0:t>버뮤다와 해외에서 이중선체 유조선을 보유·운영·용선하며 석유회사와 원유 거래업체에 서비스를 제공.</ns0:t>
+          <ns0:t>버뮤다와 해외에서 이중선체 유조선을 보유·운영·용선하며 석유회사·원유 거래업체에 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G51">
@@ -4086,7 +4086,7 @@
       </ns0:c>
       <ns0:c r="F52" t="inlineStr">
         <ns0:is>
-          <ns0:t>아시아·유럽·북미·호주에서 건화물선과 유조선을 보유·운영하며 액체·건화물 해상운송을 제공.</ns0:t>
+          <ns0:t>아시아·유럽·북미·호주에서 건화물선·유조선을 보유·운영하며 액체·건화물 해상운송 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G52">
@@ -4165,7 +4165,7 @@
       </ns0:c>
       <ns0:c r="F53" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 IT 하드웨어·소프트웨어·서비스 및 클라우드·데이터 관리 지원 솔루션 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 IT 하드웨어·소프트웨어·서비스와 클라우드·데이터 관리 지원 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G53">
@@ -4244,7 +4244,7 @@
       </ns0:c>
       <ns0:c r="F54" t="inlineStr">
         <ns0:is>
-          <ns0:t>하이브리드·퍼블릭 클라우드 부문에서 데이터 인프라용 기업 소프트웨어·시스템·서비스를 개발하는 기업.</ns0:t>
+          <ns0:t>하이브리드·퍼블릭 클라우드의 데이터 인프라용 기업 소프트웨어·시스템·서비스를 개발.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G54">
@@ -4323,7 +4323,7 @@
       </ns0:c>
       <ns0:c r="F55" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 온라인·전화·매장 및 제휴 채널을 통해 개인대출과 신용카드를 제공.</ns0:t>
+          <ns0:t>미국에서 온라인·전화·매장 및 제휴 채널을 통해 개인대출과 신용카드 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G55">
@@ -4402,7 +4402,7 @@
       </ns0:c>
       <ns0:c r="F56" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료 기술 기업으로 개인·가족·직원·소규모 단체용 건강보험과 의료 시스템용 플랫폼 제공.</ns0:t>
+          <ns0:t>미국에서 개인·가족·직원·소규모 단체용 건강보험과 의료 시스템용 플랫폼을 제공하는 의료 기술 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G56">
@@ -4481,7 +4481,7 @@
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>데이터 저장·관리 기술과 제품, 서비스를 제공하며 데이터 축소·보호·암호화 소프트웨어를 공급한다.</ns0:t>
+          <ns0:t>데이터 저장·관리 기술과 제품·서비스, 데이터 축소·보호·암호화 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57">
@@ -4560,7 +4560,7 @@
       </ns0:c>
       <ns0:c r="F58" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 재생·기존 연료를 공급하며 정유, 소매, 물류 사업을 운영한다.</ns0:t>
+          <ns0:t>미국에서 재생·기존 연료를 공급하며 정유·소매·물류 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G58">
@@ -4639,7 +4639,7 @@
       </ns0:c>
       <ns0:c r="F59" t="inlineStr">
         <ns0:is>
-          <ns0:t>선불카드, 환자 비용 부담 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
+          <ns0:t>선불카드, 환자 비용 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G59">
@@ -4718,7 +4718,7 @@
       </ns0:c>
       <ns0:c r="F60" t="inlineStr">
         <ns0:is>
-          <ns0:t>정유·물류 사업을 통해 휘발유·경유·항공유·윤활유·석유화학제품·아스팔트 등을 생산·공급하는 기업.</ns0:t>
+          <ns0:t>정유·물류 사업을 통해 휘발유·경유·항공유·윤활유·석유화학제품·아스팔트를 생산·공급한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G60">
@@ -4955,7 +4955,7 @@
       </ns0:c>
       <ns0:c r="F63" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 등에서 미드스트림·화학·정유·마케팅 및 특수제품·재생연료 사업을 운영하는 통합 다운스트림 에너지 기업.</ns0:t>
+          <ns0:t>미국 등에서 미드스트림·화학·정유·마케팅·특수제품·재생연료 사업을 운영하는 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G63">
@@ -5034,7 +5034,7 @@
       </ns0:c>
       <ns0:c r="F64" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 유조선·건화물선 사업을 운영하며 정제 석유제품 등을 운송하는 해운사.</ns0:t>
+          <ns0:t>미국과 해외에서 유조선·건화물선을 운영하며 정제 석유제품 등을 운송하는 해운사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G64">
@@ -5189,7 +5189,7 @@
       </ns0:c>
       <ns0:c r="F66" t="inlineStr">
         <ns0:is>
-          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산.</ns0:t>
+          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G66">
@@ -5268,7 +5268,7 @@
       </ns0:c>
       <ns0:c r="F67" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 생명·건강 및 자산집약형 재보험을 제공하며 장애·장기요양 관련 보장도 취급.</ns0:t>
+          <ns0:t>전 세계에서 생명·건강·자산집약형 재보험을 제공하고 장애·장기요양 관련 보장도 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G67">
@@ -5347,7 +5347,7 @@
       </ns0:c>
       <ns0:c r="F68" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 재산·상해·특종 보험과 재보험을 제공하며 재산 재해 초과손해 재보험을 취급.</ns0:t>
+          <ns0:t>미국과 해외에서 재산·상해·특종 보험 및 재보험을 제공하고 재산 재해 초과손해 재보험 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G68">
@@ -5505,7 +5505,7 @@
       </ns0:c>
       <ns0:c r="F70" t="inlineStr">
         <ns0:is>
-          <ns0:t>일본·베트남·미국·싱가포르의 미용 시술 센터에 광고·마케팅·인력관리 등 경영 서비스를 제공한다.</ns0:t>
+          <ns0:t>일본·베트남·미국·싱가포르 미용 시술 센터에 광고·마케팅·인력관리 등 경영 서비스를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G70">
@@ -5584,7 +5584,7 @@
       </ns0:c>
       <ns0:c r="F71" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
+          <ns0:t>전 세계에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G71">
@@ -5663,7 +5663,7 @@
       </ns0:c>
       <ns0:c r="F72" t="inlineStr">
         <ns0:is>
-          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청, 연료, 나프타, 윤활유, 액화석유가스 등을 공급한다.</ns0:t>
+          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청·연료·나프타·윤활유·액화석유가스를 공급한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G72">
@@ -5742,7 +5742,7 @@
       </ns0:c>
       <ns0:c r="F73" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 디지털 전환, 마케팅·미디어·커머스, 마케팅 클라우드와 커뮤니케이션 서비스 제공.</ns0:t>
+          <ns0:t>미국·영국 등에서 디지털 전환, 마케팅·미디어·커머스, 마케팅 클라우드·커뮤니케이션 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G73">
@@ -5821,7 +5821,7 @@
       </ns0:c>
       <ns0:c r="F74" t="inlineStr">
         <ns0:is>
-          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 영위하는 종합 에너지 기업.</ns0:t>
+          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 운영하는 종합 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G74">
@@ -6134,7 +6134,7 @@
       </ns0:c>
       <ns0:c r="F78" t="inlineStr">
         <ns0:is>
-          <ns0:t>그리스와 해외에서 원유·석유제품 해상 운송 서비스를 제공하며 다양한 유조선과 LNG 운반선 등을 운영.</ns0:t>
+          <ns0:t>그리스와 해외에서 원유·석유제품 해상운송을 제공하며 다양한 유조선과 LNG 운반선 등을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G78">
@@ -6213,7 +6213,7 @@
       </ns0:c>
       <ns0:c r="F79" t="inlineStr">
         <ns0:is>
-          <ns0:t>실질적인 영업활동 없이 다른 기업과의 합병·주식교환·자산인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>실질적 영업활동 없이 합병·주식교환·자산인수 등 다른 기업과의 기업결합을 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G79">
@@ -6289,7 +6289,7 @@
       </ns0:c>
       <ns0:c r="F80" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 재산·상해보험과 보증보험을 제공하며 화재·배상책임·자동차·산재보험 등을 취급.</ns0:t>
+          <ns0:t>미국에서 재산·상해·보증보험을 제공하며 화재·배상책임·자동차·산재보험 등을 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G80">
@@ -6368,7 +6368,7 @@
       </ns0:c>
       <ns0:c r="F81" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 소매·도매·구독 사업으로 의류·신발·액세서리 등 라이프스타일 상품과 서비스 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 소매·도매·구독 사업을 통해 의류·신발·액세서리 등 라이프스타일 상품·서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G81">
@@ -6447,7 +6447,7 @@
       </ns0:c>
       <ns0:c r="F82" t="inlineStr">
         <ns0:is>
-          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공.</ns0:t>
+          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G82">
@@ -6526,7 +6526,7 @@
       </ns0:c>
       <ns0:c r="F83" t="inlineStr">
         <ns0:is>
-          <ns0:t>버지니아 내 상업·개인 금융 서비스를 제공하는 은행의 지주회사로 은행 및 신탁·상속재산 서비스 운영.</ns0:t>
+          <ns0:t>버지니아에서 상업·개인 금융과 신탁·상속재산 서비스를 운영하는 은행 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G83">
@@ -6605,7 +6605,7 @@
       </ns0:c>
       <ns0:c r="F84" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계 생명과학 산업에 클라우드 소프트웨어를 제공하며 제약·바이오 기업용 CRM 제품군 등을 제공.</ns0:t>
+          <ns0:t>전 세계 생명과학 산업에 클라우드 소프트웨어와 제약·바이오 기업용 CRM 제품군 등을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G84">
@@ -6684,7 +6684,7 @@
       </ns0:c>
       <ns0:c r="F85" t="inlineStr">
         <ns0:is>
-          <ns0:t>석유 기반·저탄소 운송용 액체 연료와 석유화학 제품을 제조·판매하는 기업.</ns0:t>
+          <ns0:t>석유 기반·저탄소 운송용 액체 연료와 석유화학 제품을 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G85">
@@ -6921,7 +6921,7 @@
       </ns0:c>
       <ns0:c r="F88" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외 기업에 소비자 인텔리전스와 마케팅 자동화 소프트웨어를 제공하는 옴니채널 데이터 기반 플랫폼 운영.</ns0:t>
+          <ns0:t>미국과 해외 기업에 소비자 인텔리전스·마케팅 자동화 소프트웨어를 제공하는 옴니채널 데이터 기반 플랫폼 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G88">

</xml_diff>